<commit_message>
Add annotations and scheduled summaries
</commit_message>
<xml_diff>
--- a/examples/demo_project/01_EOAT_Audit/EOAT_Audit_Database/EOAT_Master_Tracker.xlsx
+++ b/examples/demo_project/01_EOAT_Audit/EOAT_Audit_Database/EOAT_Master_Tracker.xlsx
@@ -15,8 +15,12 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FMEA Draft" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Action Items" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Photo Index" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit by Press" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'EOAT Inventory'!$A$1:$BI$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Audit by Press'!$A$3:$Q$3</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -24,7 +28,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -32,16 +36,49 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="00666666"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001F1F1F"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F4E78"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9EAF7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00BDD7EE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFFFF"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -49,12 +86,32 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <bottom style="thin">
+        <color rgb="00D9E2F3"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -420,8 +477,30 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BA4"/>
+  <dimension ref="A1:BI4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="13" customWidth="1" min="12" max="12"/>
+    <col width="13" customWidth="1" min="13" max="13"/>
+    <col width="13" customWidth="1" min="14" max="14"/>
+    <col width="13" customWidth="1" min="15" max="15"/>
+    <col width="13" customWidth="1" min="16" max="16"/>
+    <col width="13" customWidth="1" min="17" max="17"/>
+    <col width="13" customWidth="1" min="18" max="18"/>
+    <col width="13" customWidth="1" min="19" max="19"/>
+    <col width="13" customWidth="1" min="20" max="20"/>
+    <col width="13" customWidth="1" min="22" max="22"/>
+    <col width="13" customWidth="1" min="23" max="23"/>
+    <col width="13" customWidth="1" min="24" max="24"/>
+    <col width="13" customWidth="1" min="25" max="25"/>
+    <col width="13" customWidth="1" min="26" max="26"/>
+    <col width="13" customWidth="1" min="30" max="30"/>
+    <col width="13" customWidth="1" min="31" max="31"/>
+    <col width="13" customWidth="1" min="58" max="58"/>
+    <col width="13" customWidth="1" min="59" max="59"/>
+    <col width="13" customWidth="1" min="60" max="60"/>
+    <col width="13" customWidth="1" min="61" max="61"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -486,207 +565,247 @@
       </c>
       <c r="M1" t="inlineStr">
         <is>
+          <t>EOAT Moves</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
           <t>Connection Type</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>Number of Parts Picked</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t># of Grippers</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>Gripper Type</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>Gripper Model</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>Gripper Size</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
         <is>
           <t>Cup Type/Material</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>Cup Diameter/Size</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
-        <is>
-          <t>Gripper Model</t>
-        </is>
-      </c>
-      <c r="Q1" t="inlineStr">
-        <is>
-          <t>Gripper Size</t>
-        </is>
-      </c>
-      <c r="R1" t="inlineStr">
-        <is>
-          <t>Number of Vacuum Cups</t>
-        </is>
-      </c>
-      <c r="S1" t="inlineStr">
-        <is>
-          <t>Gripper Type</t>
-        </is>
-      </c>
-      <c r="T1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>Vacuum Generator Type</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
-        <is>
-          <t>Vacuum Zones</t>
-        </is>
-      </c>
-      <c r="V1" t="inlineStr">
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>EOAT Vacuum Circuits</t>
+        </is>
+      </c>
+      <c r="X1" t="inlineStr">
+        <is>
+          <t>EOAT Pressure Circuits</t>
+        </is>
+      </c>
+      <c r="Y1" t="inlineStr">
+        <is>
+          <t>EOAT Interchangeable Circuits</t>
+        </is>
+      </c>
+      <c r="Z1" t="inlineStr">
         <is>
           <t>Sensors Present?</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t>Sensor Type</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="AB1" t="inlineStr">
         <is>
           <t>Sensor Brand/Model</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="AC1" t="inlineStr">
         <is>
           <t>Vacuum Confirmation Present?</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="AD1" t="inlineStr">
         <is>
           <t>Part-Present Detection Present?</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AE1" t="inlineStr">
+        <is>
+          <t>Electrical/Wiring Present?</t>
+        </is>
+      </c>
+      <c r="AF1" t="inlineStr">
         <is>
           <t>Quick Disconnects Present?</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AG1" t="inlineStr">
         <is>
           <t>Pneumatic Quick Disconnect Type</t>
         </is>
       </c>
-      <c r="AC1" t="inlineStr">
+      <c r="AH1" t="inlineStr">
         <is>
           <t>Electrical Quick Disconnect Type</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr">
+      <c r="AI1" t="inlineStr">
         <is>
           <t>Tubing Condition</t>
         </is>
       </c>
-      <c r="AE1" t="inlineStr">
+      <c r="AJ1" t="inlineStr">
         <is>
           <t>Tubing Routing Notes</t>
         </is>
       </c>
-      <c r="AF1" t="inlineStr">
+      <c r="AK1" t="inlineStr">
         <is>
           <t>Cable Management Condition</t>
         </is>
       </c>
-      <c r="AG1" t="inlineStr">
+      <c r="AL1" t="inlineStr">
         <is>
           <t>Mounting Hardware Condition</t>
         </is>
       </c>
-      <c r="AH1" t="inlineStr">
+      <c r="AM1" t="inlineStr">
         <is>
           <t>EOAT Alignment Condition</t>
         </is>
       </c>
-      <c r="AI1" t="inlineStr">
+      <c r="AN1" t="inlineStr">
         <is>
           <t>Fastener/Locking Hardware Present?</t>
         </is>
       </c>
-      <c r="AJ1" t="inlineStr">
+      <c r="AO1" t="inlineStr">
         <is>
           <t>Estimated EOAT Weight</t>
         </is>
       </c>
-      <c r="AK1" t="inlineStr">
+      <c r="AP1" t="inlineStr">
         <is>
           <t>Known Issues</t>
         </is>
       </c>
-      <c r="AL1" t="inlineStr">
+      <c r="AQ1" t="inlineStr">
         <is>
           <t>Drop/Mis-Pick History</t>
         </is>
       </c>
-      <c r="AM1" t="inlineStr">
+      <c r="AR1" t="inlineStr">
         <is>
           <t>Maintenance Frequency</t>
         </is>
       </c>
-      <c r="AN1" t="inlineStr">
+      <c r="AS1" t="inlineStr">
         <is>
           <t>Cycle Time Concern?</t>
         </is>
       </c>
-      <c r="AO1" t="inlineStr">
+      <c r="AT1" t="inlineStr">
         <is>
           <t>Scrap/Quality Concern?</t>
         </is>
       </c>
-      <c r="AP1" t="inlineStr">
+      <c r="AU1" t="inlineStr">
         <is>
           <t>Changeover Difficulty</t>
         </is>
       </c>
-      <c r="AQ1" t="inlineStr">
+      <c r="AV1" t="inlineStr">
         <is>
           <t>Spare Parts Identified?</t>
         </is>
       </c>
-      <c r="AR1" t="inlineStr">
+      <c r="AW1" t="inlineStr">
         <is>
           <t>Drawing/CAD Available?</t>
         </is>
       </c>
-      <c r="AS1" t="inlineStr">
+      <c r="AX1" t="inlineStr">
         <is>
           <t>BOM Available?</t>
         </is>
       </c>
-      <c r="AT1" t="inlineStr">
+      <c r="AY1" t="inlineStr">
         <is>
           <t>Process Binder Complete?</t>
         </is>
       </c>
-      <c r="AU1" t="inlineStr">
+      <c r="AZ1" t="inlineStr">
         <is>
           <t>Photos Taken?</t>
         </is>
       </c>
-      <c r="AV1" t="inlineStr">
+      <c r="BA1" t="inlineStr">
         <is>
           <t>Photo Folder/Link</t>
         </is>
       </c>
-      <c r="AW1" t="inlineStr">
+      <c r="BB1" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="AX1" t="inlineStr">
+      <c r="BC1" t="inlineStr">
         <is>
           <t>Priority</t>
         </is>
       </c>
-      <c r="AY1" t="inlineStr">
+      <c r="BD1" t="inlineStr">
         <is>
           <t>Pilot Candidate?</t>
         </is>
       </c>
-      <c r="AZ1" t="inlineStr">
+      <c r="BE1" t="inlineStr">
         <is>
           <t>Follow-Up Needed</t>
         </is>
       </c>
-      <c r="BA1" t="inlineStr">
+      <c r="BF1" t="inlineStr">
         <is>
           <t>Notes</t>
+        </is>
+      </c>
+      <c r="BG1" t="inlineStr">
+        <is>
+          <t>Entry Type</t>
+        </is>
+      </c>
+      <c r="BH1" t="inlineStr">
+        <is>
+          <t>Source Audit ID</t>
+        </is>
+      </c>
+      <c r="BI1" t="inlineStr">
+        <is>
+          <t>Compatibility Source</t>
         </is>
       </c>
     </row>
@@ -751,185 +870,195 @@
           <t>Vacuum</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr"/>
-      <c r="N2" t="inlineStr">
+      <c r="O2" t="n">
+        <v>8</v>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
         <is>
           <t>Nitrile bellows cup</t>
         </is>
       </c>
-      <c r="O2" t="inlineStr">
+      <c r="U2" t="inlineStr">
         <is>
           <t>20 mm</t>
         </is>
       </c>
-      <c r="P2" t="inlineStr"/>
-      <c r="Q2" t="inlineStr"/>
-      <c r="R2" t="n">
-        <v>8</v>
-      </c>
-      <c r="S2" t="inlineStr"/>
-      <c r="T2" t="inlineStr">
+      <c r="V2" t="inlineStr">
         <is>
           <t>Venturi</t>
         </is>
       </c>
-      <c r="U2" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="V2" t="inlineStr">
+      <c r="Z2" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="W2" t="inlineStr">
+      <c r="AA2" t="inlineStr">
         <is>
           <t>Vacuum switch</t>
         </is>
       </c>
-      <c r="X2" t="inlineStr">
+      <c r="AB2" t="inlineStr">
         <is>
           <t>SMC ZSE20</t>
         </is>
       </c>
-      <c r="Y2" t="inlineStr">
+      <c r="AC2" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="Z2" t="inlineStr">
+      <c r="AD2" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="AA2" t="inlineStr">
+      <c r="AE2" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="AB2" t="inlineStr">
+      <c r="AF2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AG2" t="inlineStr">
         <is>
           <t>Push-to-connect</t>
         </is>
       </c>
-      <c r="AC2" t="inlineStr">
+      <c r="AH2" t="inlineStr">
         <is>
           <t>M12</t>
         </is>
       </c>
-      <c r="AD2" t="inlineStr">
+      <c r="AI2" t="inlineStr">
         <is>
           <t>Leaking</t>
         </is>
       </c>
-      <c r="AE2" t="inlineStr">
+      <c r="AJ2" t="inlineStr">
         <is>
           <t>Tubing wear near wrist rotation.</t>
         </is>
       </c>
-      <c r="AF2" t="inlineStr">
+      <c r="AK2" t="inlineStr">
         <is>
           <t>Loose</t>
         </is>
       </c>
-      <c r="AG2" t="inlineStr">
+      <c r="AL2" t="inlineStr">
         <is>
           <t>Good</t>
         </is>
       </c>
-      <c r="AH2" t="inlineStr">
+      <c r="AM2" t="inlineStr">
         <is>
           <t>Needs verification</t>
         </is>
       </c>
-      <c r="AI2" t="inlineStr">
+      <c r="AN2" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="AJ2" t="inlineStr"/>
-      <c r="AK2" t="inlineStr">
+      <c r="AP2" t="inlineStr">
         <is>
           <t>Vacuum loss; part drops; tubing wear</t>
         </is>
       </c>
-      <c r="AL2" t="inlineStr">
+      <c r="AQ2" t="inlineStr">
         <is>
           <t>Recurring part drops on startup.</t>
         </is>
       </c>
-      <c r="AM2" t="inlineStr">
+      <c r="AR2" t="inlineStr">
         <is>
           <t>Weekly</t>
         </is>
       </c>
-      <c r="AN2" t="inlineStr">
+      <c r="AS2" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="AO2" t="inlineStr">
+      <c r="AT2" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="AP2" t="inlineStr">
+      <c r="AU2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="AQ2" t="inlineStr">
+      <c r="AV2" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="AR2" t="inlineStr">
+      <c r="AW2" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="AS2" t="inlineStr">
+      <c r="AX2" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="AT2" t="inlineStr">
+      <c r="AY2" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="AU2" t="inlineStr">
+      <c r="AZ2" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="AV2" t="inlineStr">
+      <c r="BA2" t="inlineStr">
         <is>
           <t>01_EOAT_Audit/Cell_Photos/Overall</t>
         </is>
       </c>
-      <c r="AW2" t="inlineStr">
+      <c r="BB2" t="inlineStr">
         <is>
           <t>Candidate for pilot</t>
         </is>
       </c>
-      <c r="AX2" t="inlineStr">
+      <c r="BC2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="AY2" t="inlineStr">
+      <c r="BD2" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="AZ2" t="inlineStr">
+      <c r="BE2" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="BA2" t="inlineStr">
+      <c r="BF2" t="inlineStr">
         <is>
           <t>Known issue cell with strong pilot potential.</t>
         </is>
@@ -986,125 +1115,117 @@
           <t>Gripper EOAT family B sample</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr"/>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Mechanical gripper</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr"/>
-      <c r="N3" t="inlineStr"/>
-      <c r="O3" t="inlineStr"/>
-      <c r="P3" t="inlineStr"/>
-      <c r="Q3" t="inlineStr"/>
-      <c r="R3" t="inlineStr"/>
-      <c r="S3" t="inlineStr">
-        <is>
-          <t>Parallel jaw</t>
-        </is>
-      </c>
-      <c r="T3" t="inlineStr"/>
-      <c r="U3" t="inlineStr"/>
-      <c r="V3" t="inlineStr">
+          <t>Mechanical / Gripper</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>Single Pressure</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>MHZL2-10S</t>
+        </is>
+      </c>
+      <c r="Z3" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="W3" t="inlineStr">
+      <c r="AA3" t="inlineStr">
         <is>
           <t>Part-present sensor</t>
         </is>
       </c>
-      <c r="X3" t="inlineStr"/>
-      <c r="Y3" t="inlineStr"/>
-      <c r="Z3" t="inlineStr"/>
-      <c r="AA3" t="inlineStr"/>
-      <c r="AB3" t="inlineStr"/>
-      <c r="AC3" t="inlineStr"/>
-      <c r="AD3" t="inlineStr">
+      <c r="AE3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AI3" t="inlineStr">
         <is>
           <t>Good</t>
         </is>
       </c>
-      <c r="AE3" t="inlineStr"/>
-      <c r="AF3" t="inlineStr">
+      <c r="AK3" t="inlineStr">
         <is>
           <t>Good</t>
         </is>
       </c>
-      <c r="AG3" t="inlineStr">
+      <c r="AL3" t="inlineStr">
         <is>
           <t>Good</t>
         </is>
       </c>
-      <c r="AH3" t="inlineStr">
+      <c r="AM3" t="inlineStr">
         <is>
           <t>Good</t>
         </is>
       </c>
-      <c r="AI3" t="inlineStr"/>
-      <c r="AJ3" t="inlineStr"/>
-      <c r="AK3" t="inlineStr">
+      <c r="AP3" t="inlineStr">
         <is>
           <t>Sensor failure during intermittent cable flex.</t>
         </is>
       </c>
-      <c r="AL3" t="inlineStr"/>
-      <c r="AM3" t="inlineStr">
+      <c r="AR3" t="inlineStr">
         <is>
           <t>Monthly</t>
         </is>
       </c>
-      <c r="AN3" t="inlineStr"/>
-      <c r="AO3" t="inlineStr"/>
-      <c r="AP3" t="inlineStr"/>
-      <c r="AQ3" t="inlineStr">
+      <c r="AV3" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="AR3" t="inlineStr">
+      <c r="AW3" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="AS3" t="inlineStr">
+      <c r="AX3" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="AT3" t="inlineStr">
+      <c r="AY3" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="AU3" t="inlineStr">
+      <c r="AZ3" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="AV3" t="inlineStr"/>
-      <c r="AW3" t="inlineStr">
+      <c r="BB3" t="inlineStr">
         <is>
           <t>Audited</t>
         </is>
       </c>
-      <c r="AX3" t="inlineStr">
+      <c r="BC3" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="AY3" t="inlineStr">
+      <c r="BD3" t="inlineStr">
         <is>
           <t>Maybe</t>
         </is>
       </c>
-      <c r="AZ3" t="inlineStr">
+      <c r="BE3" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="BA3" t="inlineStr">
+      <c r="BF3" t="inlineStr">
         <is>
           <t>Missing documentation fields are intentional fake data.</t>
         </is>
@@ -1161,137 +1282,182 @@
           <t>Hybrid EOAT family C sample</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr"/>
       <c r="L4" t="inlineStr">
         <is>
           <t>Hybrid</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr"/>
-      <c r="N4" t="inlineStr">
+      <c r="O4" t="n">
+        <v>4</v>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>Double Pressure</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>MHZL2-16D</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
         <is>
           <t>Silicone flat cup</t>
         </is>
       </c>
-      <c r="O4" t="inlineStr"/>
-      <c r="P4" t="inlineStr"/>
-      <c r="Q4" t="inlineStr"/>
-      <c r="R4" t="n">
-        <v>4</v>
-      </c>
-      <c r="S4" t="inlineStr">
-        <is>
-          <t>Clamp assist</t>
-        </is>
-      </c>
-      <c r="T4" t="inlineStr"/>
-      <c r="U4" t="inlineStr"/>
-      <c r="V4" t="inlineStr">
+      <c r="Z4" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="W4" t="inlineStr">
+      <c r="AA4" t="inlineStr">
         <is>
           <t>Vacuum and part-present</t>
         </is>
       </c>
-      <c r="X4" t="inlineStr"/>
-      <c r="Y4" t="inlineStr"/>
-      <c r="Z4" t="inlineStr"/>
-      <c r="AA4" t="inlineStr"/>
-      <c r="AB4" t="inlineStr"/>
-      <c r="AC4" t="inlineStr"/>
-      <c r="AD4" t="inlineStr">
+      <c r="AE4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AI4" t="inlineStr">
         <is>
           <t>Fair</t>
         </is>
       </c>
-      <c r="AE4" t="inlineStr"/>
-      <c r="AF4" t="inlineStr">
+      <c r="AK4" t="inlineStr">
         <is>
           <t>Good</t>
         </is>
       </c>
-      <c r="AG4" t="inlineStr">
+      <c r="AL4" t="inlineStr">
         <is>
           <t>Good</t>
         </is>
       </c>
-      <c r="AH4" t="inlineStr">
+      <c r="AM4" t="inlineStr">
         <is>
           <t>Good</t>
         </is>
       </c>
-      <c r="AI4" t="inlineStr"/>
-      <c r="AJ4" t="inlineStr"/>
-      <c r="AK4" t="inlineStr">
+      <c r="AP4" t="inlineStr">
         <is>
           <t>Cable management issue previously corrected.</t>
         </is>
       </c>
-      <c r="AL4" t="inlineStr"/>
-      <c r="AM4" t="inlineStr">
+      <c r="AR4" t="inlineStr">
         <is>
           <t>Monthly</t>
         </is>
       </c>
-      <c r="AN4" t="inlineStr"/>
-      <c r="AO4" t="inlineStr"/>
-      <c r="AP4" t="inlineStr"/>
-      <c r="AQ4" t="inlineStr">
+      <c r="AV4" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="AR4" t="inlineStr">
+      <c r="AW4" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="AS4" t="inlineStr">
+      <c r="AX4" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="AT4" t="inlineStr">
+      <c r="AY4" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="AU4" t="inlineStr">
+      <c r="AZ4" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="AV4" t="inlineStr"/>
-      <c r="AW4" t="inlineStr">
+      <c r="BB4" t="inlineStr">
         <is>
           <t>Audited</t>
         </is>
       </c>
-      <c r="AX4" t="inlineStr">
+      <c r="BC4" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="AY4" t="inlineStr">
+      <c r="BD4" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="AZ4" t="inlineStr">
+      <c r="BE4" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="BA4" t="inlineStr">
+      <c r="BF4" t="inlineStr">
         <is>
           <t>Complete documentation control row.</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:BI1"/>
+  <dataValidations count="16">
+    <dataValidation sqref="S2:S1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid circuit count" error="Enter a non-negative whole number, or leave blank if not known yet." promptTitle="Circuit count" prompt="Use a non-negative whole number." type="whole" operator="greaterThanOrEqual">
+      <formula1>0</formula1>
+    </dataValidation>
+    <dataValidation sqref="AF2:AF1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Choose a value from the dropdown list." promptTitle="Dropdown" prompt="Choose a standard value, or leave blank if not known yet." type="list">
+      <formula1>"Yes,No,Unknown / Not Checked,N/A"</formula1>
+    </dataValidation>
+    <dataValidation sqref="BH2:BH1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Choose a value from the dropdown list." promptTitle="Dropdown" prompt="Choose a standard value, or leave blank if not known yet." type="list">
+      <formula1>"Audited,Compatible"</formula1>
+    </dataValidation>
+    <dataValidation sqref="Z2:Z1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid whole number" error="Enter a non-negative whole number, or leave blank if not known yet." promptTitle="Whole number" prompt="Use a non-negative whole number." type="whole" operator="greaterThanOrEqual">
+      <formula1>0</formula1>
+    </dataValidation>
+    <dataValidation sqref="L2:L1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Choose a value from the dropdown list." promptTitle="Dropdown" prompt="Choose a standard value, or leave blank if not known yet." type="list">
+      <formula1>"Vacuum,Mechanical / Gripper,Hybrid,Unknown / Needs Review,Miscellaneous,N/A"</formula1>
+    </dataValidation>
+    <dataValidation sqref="M2:M1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Choose a value from the dropdown list." promptTitle="Dropdown" prompt="Choose a standard value, or leave blank if not known yet." type="list">
+      <formula1>"Part,Sprue,Both"</formula1>
+    </dataValidation>
+    <dataValidation sqref="N2:N1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Choose a value from the dropdown list." promptTitle="Dropdown" prompt="Choose a standard value, or leave blank if not known yet." type="list">
+      <formula1>"ATI,DoveTail,Direct Mount,Lever Lock,N/A"</formula1>
+    </dataValidation>
+    <dataValidation sqref="Q2:Q1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Choose a value from the dropdown list." promptTitle="Dropdown" prompt="Choose a standard value, or leave blank if not known yet." type="list">
+      <formula1>"Single Pressure,Double Pressure,N/A"</formula1>
+    </dataValidation>
+    <dataValidation sqref="K2:K1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Choose a value from the dropdown list." promptTitle="Dropdown" prompt="Choose a standard value, or leave blank if not known yet." type="list">
+      <formula1>"Cleanroom,Non-Cleanroom,Whiteroom,Unknown / Not Checked,N/A"</formula1>
+    </dataValidation>
+    <dataValidation sqref="AE2:AE1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Choose a value from the dropdown list." promptTitle="Dropdown" prompt="Choose a standard value, or leave blank if not known yet." type="list">
+      <formula1>"Yes,No,Unknown / Not Checked,N/A"</formula1>
+    </dataValidation>
+    <dataValidation sqref="BG2:BG1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Choose a value from the dropdown list." promptTitle="Dropdown" prompt="Choose a standard value, or leave blank if not known yet." type="list">
+      <formula1>"Audited,Compatible"</formula1>
+    </dataValidation>
+    <dataValidation sqref="O2:O1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid whole number" error="Enter a non-negative whole number, or leave blank if not known yet." promptTitle="Whole number" prompt="Use a non-negative whole number." type="whole" operator="greaterThanOrEqual">
+      <formula1>0</formula1>
+    </dataValidation>
+    <dataValidation sqref="P2:P1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid whole number" error="Enter a non-negative whole number, or leave blank if not known yet." promptTitle="Whole number" prompt="Use a non-negative whole number." type="whole" operator="greaterThanOrEqual">
+      <formula1>0</formula1>
+    </dataValidation>
+    <dataValidation sqref="X2:X1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid whole number" error="Enter a non-negative whole number, or leave blank if not known yet." promptTitle="Whole number" prompt="Use a non-negative whole number." type="whole" operator="greaterThanOrEqual">
+      <formula1>0</formula1>
+    </dataValidation>
+    <dataValidation sqref="W2:W1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid whole number" error="Enter a non-negative whole number, or leave blank if not known yet." promptTitle="Whole number" prompt="Use a non-negative whole number." type="whole" operator="greaterThanOrEqual">
+      <formula1>0</formula1>
+    </dataValidation>
+    <dataValidation sqref="Y2:Y1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid whole number" error="Enter a non-negative whole number, or leave blank if not known yet." promptTitle="Whole number" prompt="Use a non-negative whole number." type="whole" operator="greaterThanOrEqual">
+      <formula1>0</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1559,18 +1725,11 @@
           <t>Mis-picks</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr"/>
-      <c r="M3" t="inlineStr"/>
-      <c r="N3" t="inlineStr"/>
-      <c r="O3" t="inlineStr"/>
-      <c r="P3" t="inlineStr"/>
-      <c r="Q3" t="inlineStr"/>
       <c r="R3" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="S3" t="inlineStr"/>
       <c r="T3" t="inlineStr">
         <is>
           <t>Missing risk numbers are intentional.</t>
@@ -1618,9 +1777,6 @@
           <t>Tubing rubs on bracket.</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
       <c r="L4" t="n">
         <v>5</v>
       </c>
@@ -1630,16 +1786,11 @@
       <c r="N4" t="n">
         <v>5</v>
       </c>
-      <c r="O4" t="inlineStr"/>
-      <c r="P4" t="inlineStr"/>
-      <c r="Q4" t="inlineStr"/>
       <c r="R4" t="inlineStr">
         <is>
           <t>In progress</t>
         </is>
       </c>
-      <c r="S4" t="inlineStr"/>
-      <c r="T4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1811,13 +1962,11 @@
       <c r="O2" t="n">
         <v>3</v>
       </c>
-      <c r="P2" t="inlineStr"/>
       <c r="Q2" t="inlineStr">
         <is>
           <t>Fake MES extract</t>
         </is>
       </c>
-      <c r="R2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1872,20 +2021,17 @@
       <c r="L3" t="n">
         <v>4</v>
       </c>
-      <c r="M3" t="inlineStr"/>
       <c r="N3" t="n">
         <v>21</v>
       </c>
       <c r="O3" t="n">
         <v>2</v>
       </c>
-      <c r="P3" t="inlineStr"/>
       <c r="Q3" t="inlineStr">
         <is>
           <t>Fake shift notes</t>
         </is>
       </c>
-      <c r="R3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1898,26 +2044,11 @@
           <t>2026-05-18</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr">
         <is>
           <t>Press 103</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr"/>
-      <c r="N4" t="inlineStr"/>
-      <c r="O4" t="inlineStr"/>
-      <c r="P4" t="inlineStr"/>
-      <c r="Q4" t="inlineStr"/>
-      <c r="R4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2429,13 +2560,11 @@
           <t>Maintenance</t>
         </is>
       </c>
-      <c r="O2" t="inlineStr"/>
       <c r="P2" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="Q2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -2473,20 +2602,11 @@
           <t>Cable flex</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
-      <c r="L3" t="inlineStr"/>
-      <c r="M3" t="inlineStr"/>
-      <c r="N3" t="inlineStr"/>
-      <c r="O3" t="inlineStr"/>
       <c r="P3" t="inlineStr">
         <is>
           <t>Draft</t>
         </is>
       </c>
-      <c r="Q3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2595,7 +2715,6 @@
           <t>In progress</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr">
         <is>
           <t>Carryover action item for morning plan.</t>
@@ -2719,7 +2838,6 @@
           <t>AUD-20260518-001</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
           <t>Seed row.</t>
@@ -2729,4 +2847,453 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:Q9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="34" customWidth="1" min="13" max="13"/>
+    <col width="28" customWidth="1" min="14" max="14"/>
+    <col width="18" customWidth="1" min="15" max="15"/>
+    <col width="18" customWidth="1" min="16" max="16"/>
+    <col width="18" customWidth="1" min="17" max="17"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>EOAT Audit by Press</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="n"/>
+      <c r="C1" s="1" t="n"/>
+      <c r="D1" s="1" t="n"/>
+      <c r="E1" s="1" t="n"/>
+      <c r="F1" s="1" t="n"/>
+      <c r="G1" s="1" t="n"/>
+      <c r="H1" s="1" t="n"/>
+      <c r="I1" s="1" t="n"/>
+      <c r="J1" s="1" t="n"/>
+      <c r="K1" s="1" t="n"/>
+      <c r="L1" s="1" t="n"/>
+      <c r="M1" s="1" t="n"/>
+      <c r="N1" s="1" t="n"/>
+      <c r="O1" s="1" t="n"/>
+      <c r="P1" s="1" t="n"/>
+      <c r="Q1" s="1" t="n"/>
+    </row>
+    <row r="2" ht="20" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Last refreshed: 2026-05-27 16:02</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="n"/>
+      <c r="C2" s="2" t="n"/>
+      <c r="D2" s="2" t="n"/>
+      <c r="E2" s="2" t="n"/>
+      <c r="F2" s="2" t="n"/>
+      <c r="G2" s="2" t="n"/>
+      <c r="H2" s="2" t="n"/>
+      <c r="I2" s="2" t="n"/>
+      <c r="J2" s="2" t="n"/>
+      <c r="K2" s="2" t="n"/>
+      <c r="L2" s="2" t="n"/>
+      <c r="M2" s="2" t="n"/>
+      <c r="N2" s="2" t="n"/>
+      <c r="O2" s="2" t="n"/>
+      <c r="P2" s="2" t="n"/>
+      <c r="Q2" s="2" t="inlineStr">
+        <is>
+          <t>Generated view from EOAT Inventory</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="32" customHeight="1">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Audit ID</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Auditor</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>Plant/Area</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>Press/Machine #</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>Tool #</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>Robot Type</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>EOAT Type</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>EOAT Moves</t>
+        </is>
+      </c>
+      <c r="J3" s="3" t="inlineStr">
+        <is>
+          <t>Connection Type</t>
+        </is>
+      </c>
+      <c r="K3" s="3" t="inlineStr">
+        <is>
+          <t>Cleanroom/Non-Cleanroom</t>
+        </is>
+      </c>
+      <c r="L3" s="3" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="M3" s="3" t="inlineStr">
+        <is>
+          <t>Entry Type</t>
+        </is>
+      </c>
+      <c r="N3" s="3" t="inlineStr">
+        <is>
+          <t>Source Audit ID</t>
+        </is>
+      </c>
+      <c r="O3" s="3" t="inlineStr">
+        <is>
+          <t>Priority</t>
+        </is>
+      </c>
+      <c r="P3" s="3" t="inlineStr">
+        <is>
+          <t>Known Issues / Observations</t>
+        </is>
+      </c>
+      <c r="Q3" s="3" t="inlineStr">
+        <is>
+          <t>Photo Link / Photo Count</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" collapsed="1" ht="20" customHeight="1">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Molding / Press 101 - 1 physical, 0 compatible, 1 total entry</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="n"/>
+      <c r="C4" s="4" t="n"/>
+      <c r="D4" s="4" t="n"/>
+      <c r="E4" s="4" t="n"/>
+      <c r="F4" s="4" t="n"/>
+      <c r="G4" s="4" t="n"/>
+      <c r="H4" s="4" t="n"/>
+      <c r="I4" s="4" t="n"/>
+      <c r="J4" s="4" t="n"/>
+      <c r="K4" s="4" t="n"/>
+      <c r="L4" s="4" t="n"/>
+      <c r="M4" s="4" t="n"/>
+      <c r="N4" s="4" t="n"/>
+      <c r="O4" s="4" t="n"/>
+      <c r="P4" s="4" t="n"/>
+      <c r="Q4" s="4" t="inlineStr">
+        <is>
+          <t>1 physical / 0 compatible / 1 total</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" hidden="1" outlineLevel="1" ht="20" customHeight="1">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>AUD-20260518-001</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>Fake Intern</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>Molding</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>Press 101</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>TOOL-A</t>
+        </is>
+      </c>
+      <c r="G5" s="5" t="inlineStr">
+        <is>
+          <t>Wittmann R9</t>
+        </is>
+      </c>
+      <c r="H5" s="5" t="inlineStr">
+        <is>
+          <t>Vacuum</t>
+        </is>
+      </c>
+      <c r="I5" s="5" t="n"/>
+      <c r="J5" s="5" t="n"/>
+      <c r="K5" s="5" t="inlineStr">
+        <is>
+          <t>Non-cleanroom</t>
+        </is>
+      </c>
+      <c r="L5" s="5" t="inlineStr">
+        <is>
+          <t>Candidate for pilot</t>
+        </is>
+      </c>
+      <c r="M5" s="5" t="n"/>
+      <c r="N5" s="5" t="n"/>
+      <c r="O5" s="5" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="P5" s="5" t="inlineStr">
+        <is>
+          <t>Vacuum loss; part drops; tubing wear</t>
+        </is>
+      </c>
+      <c r="Q5" s="5" t="inlineStr">
+        <is>
+          <t>01_EOAT_Audit/Cell_Photos/Overall</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" collapsed="1" ht="20" customHeight="1">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Molding / Press 102 - 1 physical, 0 compatible, 1 total entry</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="n"/>
+      <c r="C6" s="4" t="n"/>
+      <c r="D6" s="4" t="n"/>
+      <c r="E6" s="4" t="n"/>
+      <c r="F6" s="4" t="n"/>
+      <c r="G6" s="4" t="n"/>
+      <c r="H6" s="4" t="n"/>
+      <c r="I6" s="4" t="n"/>
+      <c r="J6" s="4" t="n"/>
+      <c r="K6" s="4" t="n"/>
+      <c r="L6" s="4" t="n"/>
+      <c r="M6" s="4" t="n"/>
+      <c r="N6" s="4" t="n"/>
+      <c r="O6" s="4" t="n"/>
+      <c r="P6" s="4" t="n"/>
+      <c r="Q6" s="4" t="inlineStr">
+        <is>
+          <t>1 physical / 0 compatible / 1 total</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" hidden="1" outlineLevel="1" ht="20" customHeight="1">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>AUD-20260518-002</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>Fake Intern</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>Molding</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>Press 102</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>TOOL-B</t>
+        </is>
+      </c>
+      <c r="G7" s="5" t="inlineStr">
+        <is>
+          <t>Engel Viper</t>
+        </is>
+      </c>
+      <c r="H7" s="5" t="inlineStr">
+        <is>
+          <t>Mechanical / Gripper</t>
+        </is>
+      </c>
+      <c r="I7" s="5" t="n"/>
+      <c r="J7" s="5" t="n"/>
+      <c r="K7" s="5" t="n"/>
+      <c r="L7" s="5" t="inlineStr">
+        <is>
+          <t>Audited</t>
+        </is>
+      </c>
+      <c r="M7" s="5" t="n"/>
+      <c r="N7" s="5" t="n"/>
+      <c r="O7" s="5" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="P7" s="5" t="inlineStr">
+        <is>
+          <t>Sensor failure during intermittent cable flex.</t>
+        </is>
+      </c>
+      <c r="Q7" s="5" t="n"/>
+    </row>
+    <row r="8" collapsed="1" ht="20" customHeight="1">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Molding / Press 103 - 1 physical, 0 compatible, 1 total entry</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="n"/>
+      <c r="C8" s="4" t="n"/>
+      <c r="D8" s="4" t="n"/>
+      <c r="E8" s="4" t="n"/>
+      <c r="F8" s="4" t="n"/>
+      <c r="G8" s="4" t="n"/>
+      <c r="H8" s="4" t="n"/>
+      <c r="I8" s="4" t="n"/>
+      <c r="J8" s="4" t="n"/>
+      <c r="K8" s="4" t="n"/>
+      <c r="L8" s="4" t="n"/>
+      <c r="M8" s="4" t="n"/>
+      <c r="N8" s="4" t="n"/>
+      <c r="O8" s="4" t="n"/>
+      <c r="P8" s="4" t="n"/>
+      <c r="Q8" s="4" t="inlineStr">
+        <is>
+          <t>1 physical / 0 compatible / 1 total</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" hidden="1" outlineLevel="1" ht="20" customHeight="1">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>AUD-20260518-003</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>Fake Intern</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>Molding</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>Press 103</t>
+        </is>
+      </c>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>TOOL-C</t>
+        </is>
+      </c>
+      <c r="G9" s="5" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="H9" s="5" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="I9" s="5" t="n"/>
+      <c r="J9" s="5" t="n"/>
+      <c r="K9" s="5" t="n"/>
+      <c r="L9" s="5" t="inlineStr">
+        <is>
+          <t>Audited</t>
+        </is>
+      </c>
+      <c r="M9" s="5" t="n"/>
+      <c r="N9" s="5" t="n"/>
+      <c r="O9" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="P9" s="5" t="inlineStr">
+        <is>
+          <t>Cable management issue previously corrected.</t>
+        </is>
+      </c>
+      <c r="Q9" s="5" t="n"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A3:Q3"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add cup count to demo master tracker workbook
</commit_message>
<xml_diff>
--- a/examples/demo_project/01_EOAT_Audit/EOAT_Audit_Database/EOAT_Master_Tracker.xlsx
+++ b/examples/demo_project/01_EOAT_Audit/EOAT_Audit_Database/EOAT_Master_Tracker.xlsx
@@ -18,7 +18,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit by Press" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'EOAT Inventory'!$A$1:$BI$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'EOAT Inventory'!$A$1:$BJ$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Audit by Press'!$A$3:$Q$3</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -477,7 +477,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BI4"/>
+  <dimension ref="A1:BJ4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="12" max="12"/>
@@ -600,210 +600,215 @@
       </c>
       <c r="T1" t="inlineStr">
         <is>
+          <t># of Cups</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
           <t>Cup Type/Material</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>Cup Diameter/Size</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>Vacuum Generator Type</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>EOAT Vacuum Circuits</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>EOAT Pressure Circuits</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>EOAT Interchangeable Circuits</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t>Sensors Present?</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AB1" t="inlineStr">
         <is>
           <t>Sensor Type</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AC1" t="inlineStr">
         <is>
           <t>Sensor Brand/Model</t>
         </is>
       </c>
-      <c r="AC1" t="inlineStr">
+      <c r="AD1" t="inlineStr">
         <is>
           <t>Vacuum Confirmation Present?</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr">
+      <c r="AE1" t="inlineStr">
         <is>
           <t>Part-Present Detection Present?</t>
         </is>
       </c>
-      <c r="AE1" t="inlineStr">
+      <c r="AF1" t="inlineStr">
         <is>
           <t>Electrical/Wiring Present?</t>
         </is>
       </c>
-      <c r="AF1" t="inlineStr">
+      <c r="AG1" t="inlineStr">
         <is>
           <t>Quick Disconnects Present?</t>
         </is>
       </c>
-      <c r="AG1" t="inlineStr">
+      <c r="AH1" t="inlineStr">
         <is>
           <t>Pneumatic Quick Disconnect Type</t>
         </is>
       </c>
-      <c r="AH1" t="inlineStr">
+      <c r="AI1" t="inlineStr">
         <is>
           <t>Electrical Quick Disconnect Type</t>
         </is>
       </c>
-      <c r="AI1" t="inlineStr">
+      <c r="AJ1" t="inlineStr">
         <is>
           <t>Tubing Condition</t>
         </is>
       </c>
-      <c r="AJ1" t="inlineStr">
+      <c r="AK1" t="inlineStr">
         <is>
           <t>Tubing Routing Notes</t>
         </is>
       </c>
-      <c r="AK1" t="inlineStr">
+      <c r="AL1" t="inlineStr">
         <is>
           <t>Cable Management Condition</t>
         </is>
       </c>
-      <c r="AL1" t="inlineStr">
+      <c r="AM1" t="inlineStr">
         <is>
           <t>Mounting Hardware Condition</t>
         </is>
       </c>
-      <c r="AM1" t="inlineStr">
+      <c r="AN1" t="inlineStr">
         <is>
           <t>EOAT Alignment Condition</t>
         </is>
       </c>
-      <c r="AN1" t="inlineStr">
+      <c r="AO1" t="inlineStr">
         <is>
           <t>Fastener/Locking Hardware Present?</t>
         </is>
       </c>
-      <c r="AO1" t="inlineStr">
+      <c r="AP1" t="inlineStr">
         <is>
           <t>Estimated EOAT Weight</t>
         </is>
       </c>
-      <c r="AP1" t="inlineStr">
+      <c r="AQ1" t="inlineStr">
         <is>
           <t>Known Issues</t>
         </is>
       </c>
-      <c r="AQ1" t="inlineStr">
+      <c r="AR1" t="inlineStr">
         <is>
           <t>Drop/Mis-Pick History</t>
         </is>
       </c>
-      <c r="AR1" t="inlineStr">
+      <c r="AS1" t="inlineStr">
         <is>
           <t>Maintenance Frequency</t>
         </is>
       </c>
-      <c r="AS1" t="inlineStr">
+      <c r="AT1" t="inlineStr">
         <is>
           <t>Cycle Time Concern?</t>
         </is>
       </c>
-      <c r="AT1" t="inlineStr">
+      <c r="AU1" t="inlineStr">
         <is>
           <t>Scrap/Quality Concern?</t>
         </is>
       </c>
-      <c r="AU1" t="inlineStr">
+      <c r="AV1" t="inlineStr">
         <is>
           <t>Changeover Difficulty</t>
         </is>
       </c>
-      <c r="AV1" t="inlineStr">
+      <c r="AW1" t="inlineStr">
         <is>
           <t>Spare Parts Identified?</t>
         </is>
       </c>
-      <c r="AW1" t="inlineStr">
+      <c r="AX1" t="inlineStr">
         <is>
           <t>Drawing/CAD Available?</t>
         </is>
       </c>
-      <c r="AX1" t="inlineStr">
+      <c r="AY1" t="inlineStr">
         <is>
           <t>BOM Available?</t>
         </is>
       </c>
-      <c r="AY1" t="inlineStr">
+      <c r="AZ1" t="inlineStr">
         <is>
           <t>Process Binder Complete?</t>
         </is>
       </c>
-      <c r="AZ1" t="inlineStr">
+      <c r="BA1" t="inlineStr">
         <is>
           <t>Photos Taken?</t>
         </is>
       </c>
-      <c r="BA1" t="inlineStr">
+      <c r="BB1" t="inlineStr">
         <is>
           <t>Photo Folder/Link</t>
         </is>
       </c>
-      <c r="BB1" t="inlineStr">
+      <c r="BC1" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="BC1" t="inlineStr">
+      <c r="BD1" t="inlineStr">
         <is>
           <t>Priority</t>
         </is>
       </c>
-      <c r="BD1" t="inlineStr">
+      <c r="BE1" t="inlineStr">
         <is>
           <t>Pilot Candidate?</t>
         </is>
       </c>
-      <c r="BE1" t="inlineStr">
+      <c r="BF1" t="inlineStr">
         <is>
           <t>Follow-Up Needed</t>
         </is>
       </c>
-      <c r="BF1" t="inlineStr">
+      <c r="BG1" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
-      <c r="BG1" t="inlineStr">
+      <c r="BH1" t="inlineStr">
         <is>
           <t>Entry Type</t>
         </is>
       </c>
-      <c r="BH1" t="inlineStr">
+      <c r="BI1" t="inlineStr">
         <is>
           <t>Source Audit ID</t>
         </is>
       </c>
-      <c r="BI1" t="inlineStr">
+      <c r="BJ1" t="inlineStr">
         <is>
           <t>Compatibility Source</t>
         </is>
@@ -888,177 +893,180 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="T2" t="inlineStr">
+      <c r="T2" t="n">
+        <v>8</v>
+      </c>
+      <c r="U2" t="inlineStr">
         <is>
           <t>Nitrile bellows cup</t>
         </is>
       </c>
-      <c r="U2" t="inlineStr">
+      <c r="V2" t="inlineStr">
         <is>
           <t>20 mm</t>
         </is>
       </c>
-      <c r="V2" t="inlineStr">
+      <c r="W2" t="inlineStr">
         <is>
           <t>Venturi</t>
         </is>
       </c>
-      <c r="Z2" t="inlineStr">
+      <c r="AA2" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="AA2" t="inlineStr">
+      <c r="AB2" t="inlineStr">
         <is>
           <t>Vacuum switch</t>
         </is>
       </c>
-      <c r="AB2" t="inlineStr">
+      <c r="AC2" t="inlineStr">
         <is>
           <t>SMC ZSE20</t>
         </is>
       </c>
-      <c r="AC2" t="inlineStr">
+      <c r="AD2" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="AD2" t="inlineStr">
+      <c r="AE2" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="AE2" t="inlineStr">
+      <c r="AF2" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="AF2" t="inlineStr">
+      <c r="AG2" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="AG2" t="inlineStr">
+      <c r="AH2" t="inlineStr">
         <is>
           <t>Push-to-connect</t>
         </is>
       </c>
-      <c r="AH2" t="inlineStr">
+      <c r="AI2" t="inlineStr">
         <is>
           <t>M12</t>
         </is>
       </c>
-      <c r="AI2" t="inlineStr">
+      <c r="AJ2" t="inlineStr">
         <is>
           <t>Leaking</t>
         </is>
       </c>
-      <c r="AJ2" t="inlineStr">
+      <c r="AK2" t="inlineStr">
         <is>
           <t>Tubing wear near wrist rotation.</t>
         </is>
       </c>
-      <c r="AK2" t="inlineStr">
+      <c r="AL2" t="inlineStr">
         <is>
           <t>Loose</t>
         </is>
       </c>
-      <c r="AL2" t="inlineStr">
+      <c r="AM2" t="inlineStr">
         <is>
           <t>Good</t>
         </is>
       </c>
-      <c r="AM2" t="inlineStr">
+      <c r="AN2" t="inlineStr">
         <is>
           <t>Needs verification</t>
         </is>
       </c>
-      <c r="AN2" t="inlineStr">
+      <c r="AO2" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="AP2" t="inlineStr">
+      <c r="AQ2" t="inlineStr">
         <is>
           <t>Vacuum loss; part drops; tubing wear</t>
         </is>
       </c>
-      <c r="AQ2" t="inlineStr">
+      <c r="AR2" t="inlineStr">
         <is>
           <t>Recurring part drops on startup.</t>
         </is>
       </c>
-      <c r="AR2" t="inlineStr">
+      <c r="AS2" t="inlineStr">
         <is>
           <t>Weekly</t>
         </is>
       </c>
-      <c r="AS2" t="inlineStr">
+      <c r="AT2" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="AT2" t="inlineStr">
+      <c r="AU2" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="AU2" t="inlineStr">
+      <c r="AV2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="AV2" t="inlineStr">
+      <c r="AW2" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="AW2" t="inlineStr">
+      <c r="AX2" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="AX2" t="inlineStr">
+      <c r="AY2" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="AY2" t="inlineStr">
+      <c r="AZ2" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="AZ2" t="inlineStr">
+      <c r="BA2" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="BA2" t="inlineStr">
+      <c r="BB2" t="inlineStr">
         <is>
           <t>01_EOAT_Audit/Cell_Photos/Overall</t>
         </is>
       </c>
-      <c r="BB2" t="inlineStr">
+      <c r="BC2" t="inlineStr">
         <is>
           <t>Candidate for pilot</t>
         </is>
       </c>
-      <c r="BC2" t="inlineStr">
+      <c r="BD2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="BD2" t="inlineStr">
+      <c r="BE2" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="BE2" t="inlineStr">
+      <c r="BF2" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="BF2" t="inlineStr">
+      <c r="BG2" t="inlineStr">
         <is>
           <t>Known issue cell with strong pilot potential.</t>
         </is>
@@ -1135,97 +1143,102 @@
           <t>MHZL2-10S</t>
         </is>
       </c>
-      <c r="Z3" t="inlineStr">
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AA3" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="AA3" t="inlineStr">
+      <c r="AB3" t="inlineStr">
         <is>
           <t>Part-present sensor</t>
         </is>
       </c>
-      <c r="AE3" t="inlineStr">
+      <c r="AF3" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="AI3" t="inlineStr">
+      <c r="AJ3" t="inlineStr">
         <is>
           <t>Good</t>
         </is>
       </c>
-      <c r="AK3" t="inlineStr">
+      <c r="AL3" t="inlineStr">
         <is>
           <t>Good</t>
         </is>
       </c>
-      <c r="AL3" t="inlineStr">
+      <c r="AM3" t="inlineStr">
         <is>
           <t>Good</t>
         </is>
       </c>
-      <c r="AM3" t="inlineStr">
+      <c r="AN3" t="inlineStr">
         <is>
           <t>Good</t>
         </is>
       </c>
-      <c r="AP3" t="inlineStr">
+      <c r="AQ3" t="inlineStr">
         <is>
           <t>Sensor failure during intermittent cable flex.</t>
         </is>
       </c>
-      <c r="AR3" t="inlineStr">
+      <c r="AS3" t="inlineStr">
         <is>
           <t>Monthly</t>
         </is>
       </c>
-      <c r="AV3" t="inlineStr">
+      <c r="AW3" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="AW3" t="inlineStr">
+      <c r="AX3" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="AX3" t="inlineStr">
+      <c r="AY3" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="AY3" t="inlineStr">
+      <c r="AZ3" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="AZ3" t="inlineStr">
+      <c r="BA3" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="BB3" t="inlineStr">
+      <c r="BC3" t="inlineStr">
         <is>
           <t>Audited</t>
         </is>
       </c>
-      <c r="BC3" t="inlineStr">
+      <c r="BD3" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="BD3" t="inlineStr">
+      <c r="BE3" t="inlineStr">
         <is>
           <t>Maybe</t>
         </is>
       </c>
-      <c r="BE3" t="inlineStr">
+      <c r="BF3" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="BF3" t="inlineStr">
+      <c r="BG3" t="inlineStr">
         <is>
           <t>Missing documentation fields are intentional fake data.</t>
         </is>
@@ -1305,120 +1318,123 @@
           <t>MHZL2-16D</t>
         </is>
       </c>
-      <c r="T4" t="inlineStr">
+      <c r="T4" t="n">
+        <v>4</v>
+      </c>
+      <c r="U4" t="inlineStr">
         <is>
           <t>Silicone flat cup</t>
         </is>
       </c>
-      <c r="Z4" t="inlineStr">
+      <c r="AA4" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="AA4" t="inlineStr">
+      <c r="AB4" t="inlineStr">
         <is>
           <t>Vacuum and part-present</t>
         </is>
       </c>
-      <c r="AE4" t="inlineStr">
+      <c r="AF4" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="AI4" t="inlineStr">
+      <c r="AJ4" t="inlineStr">
         <is>
           <t>Fair</t>
         </is>
       </c>
-      <c r="AK4" t="inlineStr">
+      <c r="AL4" t="inlineStr">
         <is>
           <t>Good</t>
         </is>
       </c>
-      <c r="AL4" t="inlineStr">
+      <c r="AM4" t="inlineStr">
         <is>
           <t>Good</t>
         </is>
       </c>
-      <c r="AM4" t="inlineStr">
+      <c r="AN4" t="inlineStr">
         <is>
           <t>Good</t>
         </is>
       </c>
-      <c r="AP4" t="inlineStr">
+      <c r="AQ4" t="inlineStr">
         <is>
           <t>Cable management issue previously corrected.</t>
         </is>
       </c>
-      <c r="AR4" t="inlineStr">
+      <c r="AS4" t="inlineStr">
         <is>
           <t>Monthly</t>
         </is>
       </c>
-      <c r="AV4" t="inlineStr">
+      <c r="AW4" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="AW4" t="inlineStr">
+      <c r="AX4" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="AX4" t="inlineStr">
+      <c r="AY4" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="AY4" t="inlineStr">
+      <c r="AZ4" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="AZ4" t="inlineStr">
+      <c r="BA4" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="BB4" t="inlineStr">
+      <c r="BC4" t="inlineStr">
         <is>
           <t>Audited</t>
         </is>
       </c>
-      <c r="BC4" t="inlineStr">
+      <c r="BD4" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="BD4" t="inlineStr">
+      <c r="BE4" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="BE4" t="inlineStr">
+      <c r="BF4" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="BF4" t="inlineStr">
+      <c r="BG4" t="inlineStr">
         <is>
           <t>Complete documentation control row.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:BI1"/>
-  <dataValidations count="16">
+  <autoFilter ref="A1:BJ1"/>
+  <dataValidations count="17">
     <dataValidation sqref="S2:S1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid circuit count" error="Enter a non-negative whole number, or leave blank if not known yet." promptTitle="Circuit count" prompt="Use a non-negative whole number." type="whole" operator="greaterThanOrEqual">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation sqref="AF2:AF1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Choose a value from the dropdown list." promptTitle="Dropdown" prompt="Choose a standard value, or leave blank if not known yet." type="list">
+    <dataValidation sqref="AE2:AE1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Choose a value from the dropdown list." promptTitle="Dropdown" prompt="Choose a standard value, or leave blank if not known yet." type="list">
       <formula1>"Yes,No,Unknown / Not Checked,N/A"</formula1>
     </dataValidation>
-    <dataValidation sqref="BH2:BH1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Choose a value from the dropdown list." promptTitle="Dropdown" prompt="Choose a standard value, or leave blank if not known yet." type="list">
+    <dataValidation sqref="BG2:BG1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Choose a value from the dropdown list." promptTitle="Dropdown" prompt="Choose a standard value, or leave blank if not known yet." type="list">
       <formula1>"Audited,Compatible"</formula1>
     </dataValidation>
-    <dataValidation sqref="Z2:Z1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid whole number" error="Enter a non-negative whole number, or leave blank if not known yet." promptTitle="Whole number" prompt="Use a non-negative whole number." type="whole" operator="greaterThanOrEqual">
+    <dataValidation sqref="W2:W1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid whole number" error="Enter a non-negative whole number, or leave blank if not known yet." promptTitle="Whole number" prompt="Use a non-negative whole number." type="whole" operator="greaterThanOrEqual">
       <formula1>0</formula1>
     </dataValidation>
     <dataValidation sqref="L2:L1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Choose a value from the dropdown list." promptTitle="Dropdown" prompt="Choose a standard value, or leave blank if not known yet." type="list">
@@ -1436,10 +1452,10 @@
     <dataValidation sqref="K2:K1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Choose a value from the dropdown list." promptTitle="Dropdown" prompt="Choose a standard value, or leave blank if not known yet." type="list">
       <formula1>"Cleanroom,Non-Cleanroom,Whiteroom,Unknown / Not Checked,N/A"</formula1>
     </dataValidation>
-    <dataValidation sqref="AE2:AE1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Choose a value from the dropdown list." promptTitle="Dropdown" prompt="Choose a standard value, or leave blank if not known yet." type="list">
+    <dataValidation sqref="AF2:AF1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Choose a value from the dropdown list." promptTitle="Dropdown" prompt="Choose a standard value, or leave blank if not known yet." type="list">
       <formula1>"Yes,No,Unknown / Not Checked,N/A"</formula1>
     </dataValidation>
-    <dataValidation sqref="BG2:BG1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Choose a value from the dropdown list." promptTitle="Dropdown" prompt="Choose a standard value, or leave blank if not known yet." type="list">
+    <dataValidation sqref="BH2:BH1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Choose a value from the dropdown list." promptTitle="Dropdown" prompt="Choose a standard value, or leave blank if not known yet." type="list">
       <formula1>"Audited,Compatible"</formula1>
     </dataValidation>
     <dataValidation sqref="O2:O1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid whole number" error="Enter a non-negative whole number, or leave blank if not known yet." promptTitle="Whole number" prompt="Use a non-negative whole number." type="whole" operator="greaterThanOrEqual">
@@ -1448,13 +1464,16 @@
     <dataValidation sqref="P2:P1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid whole number" error="Enter a non-negative whole number, or leave blank if not known yet." promptTitle="Whole number" prompt="Use a non-negative whole number." type="whole" operator="greaterThanOrEqual">
       <formula1>0</formula1>
     </dataValidation>
+    <dataValidation sqref="Y2:Y1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid whole number" error="Enter a non-negative whole number, or leave blank if not known yet." promptTitle="Whole number" prompt="Use a non-negative whole number." type="whole" operator="greaterThanOrEqual">
+      <formula1>0</formula1>
+    </dataValidation>
     <dataValidation sqref="X2:X1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid whole number" error="Enter a non-negative whole number, or leave blank if not known yet." promptTitle="Whole number" prompt="Use a non-negative whole number." type="whole" operator="greaterThanOrEqual">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation sqref="W2:W1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid whole number" error="Enter a non-negative whole number, or leave blank if not known yet." promptTitle="Whole number" prompt="Use a non-negative whole number." type="whole" operator="greaterThanOrEqual">
+    <dataValidation sqref="Z2:Z1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid whole number" error="Enter a non-negative whole number, or leave blank if not known yet." promptTitle="Whole number" prompt="Use a non-negative whole number." type="whole" operator="greaterThanOrEqual">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation sqref="Y2:Y1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid whole number" error="Enter a non-negative whole number, or leave blank if not known yet." promptTitle="Whole number" prompt="Use a non-negative whole number." type="whole" operator="greaterThanOrEqual">
+    <dataValidation sqref="T2:T1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid whole number" error="Enter a non-negative whole number, or leave blank if not known yet." promptTitle="Whole number" prompt="Use a non-negative whole number." type="whole" operator="greaterThanOrEqual">
       <formula1>0</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>